<commit_message>
Fix 9 garbled names verified from Forsyth County website
</commit_message>
<xml_diff>
--- a/Forsyth_County_Contacts.xlsx
+++ b/Forsyth_County_Contacts.xlsx
@@ -2982,12 +2982,12 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>Skip</t>
+          <t>Antoinette</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>TAo nMation Cinonetetntte Ricardo</t>
+          <t>Ricardo</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
@@ -3014,12 +3014,12 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Skip</t>
+          <t>Lauren</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>TLoa Muairn eConnt ePntulley</t>
+          <t>Pulley</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
@@ -3046,12 +3046,12 @@
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>Skip</t>
+          <t>Rachael</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>TRo aMacinh Caoneteln tNorie</t>
+          <t>Norie</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
@@ -4134,12 +4134,12 @@
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>Skip</t>
+          <t>Angel</t>
         </is>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>TAo nMagine Clo nFteinntdley</t>
+          <t>Findley</t>
         </is>
       </c>
       <c r="C117" s="2" t="inlineStr">
@@ -4166,17 +4166,17 @@
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>Skip</t>
+          <t>Georgia</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>TGo Meaoinr Cgonitaen tMiles</t>
+          <t>Miles</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>School Psychologist gmiles @forsyth.k12.ga.us</t>
+          <t>School Psychologist</t>
         </is>
       </c>
       <c r="D118" s="3" t="inlineStr">
@@ -4198,12 +4198,12 @@
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>Skip</t>
+          <t>Katie</t>
         </is>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>TKoa Mtaiine C oAntteontlli</t>
+          <t>Atolli</t>
         </is>
       </c>
       <c r="C119" s="2" t="inlineStr">
@@ -4230,12 +4230,12 @@
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>Skip</t>
+          <t>Kelli</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>TKoe Mlaliin CColnatenrti</t>
+          <t>Clari</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
@@ -5926,12 +5926,12 @@
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
         <is>
-          <t>Skip</t>
+          <t>Brian</t>
         </is>
       </c>
       <c r="B173" s="2" t="inlineStr">
         <is>
-          <t>TDo rM. aBin rCioantnen tLack</t>
+          <t>Lack</t>
         </is>
       </c>
       <c r="C173" s="2" t="inlineStr">
@@ -5958,12 +5958,12 @@
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>Skip</t>
+          <t>Tiffany</t>
         </is>
       </c>
       <c r="B174" s="2" t="inlineStr">
         <is>
-          <t>TToi Mffaainn Coyn teVntorick</t>
+          <t>Vorick</t>
         </is>
       </c>
       <c r="C174" s="2" t="inlineStr">

</xml_diff>